<commit_message>
Send the daily summary and alerts to Telegram
- telegram_report.py: summary text + gamma chart (matplotlib) via the Bot API
  (urllib, no SDK); --setup asks for the BotFather token in the terminal and
  saves telegram.json (git-ignored); every send is best-effort
- Walls/Pins/mode are read back from Excel's own calculation of GEX Calc
  (verify.excel_cells); Python totals only if Excel/the save isn't available
- notify() copies every alert to Telegram
- a workbook left open in Excel no longer aborts the run: Max Pain and GEX
  each report "Cannot save" and the run carries on to GEX and the report
  (three scheduled runs were lost to this on 2026-10-06/07)
- tests: conftest keeps tests off the real bot; format/send/chart tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GEX V.4.1.xlsx
+++ b/GEX V.4.1.xlsx
@@ -521,7 +521,7 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'GEX Calc'!$A$2:$A$124</f>
+              <f>'GEX Calc'!$A$2:$A$84</f>
               <numCache>
                 <formatCode>#,##0</formatCode>
                 <ptCount val="61"/>
@@ -713,7 +713,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'GEX Calc'!$C$2:$C$124</f>
+              <f>'GEX Calc'!$C$2:$C$84</f>
               <numCache>
                 <formatCode>#,##0</formatCode>
                 <ptCount val="61"/>
@@ -1390,7 +1390,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -1445,7 +1445,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -1456,7 +1456,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1522,7 +1522,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1533,7 +1533,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1555,7 +1555,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1566,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1577,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -1599,7 +1599,7 @@
         <v>0</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -1610,7 +1610,7 @@
         <v>0</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>60</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1643,7 +1643,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
@@ -1662,10 +1662,10 @@
         <v>4125</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -1687,7 +1687,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -1695,10 +1695,10 @@
         <v>4140</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -1709,7 +1709,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -1720,7 +1720,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>72</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -1731,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -1739,10 +1739,10 @@
         <v>4160</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -1753,7 +1753,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -1761,10 +1761,10 @@
         <v>4170</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -1772,10 +1772,10 @@
         <v>4175</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -1783,10 +1783,10 @@
         <v>4180</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -1797,7 +1797,7 @@
         <v>2</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -1808,7 +1808,7 @@
         <v>0</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -1816,10 +1816,10 @@
         <v>4195</v>
       </c>
       <c r="B42" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C42" s="3" t="n">
         <v>1</v>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
@@ -1827,10 +1827,10 @@
         <v>4200</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>96</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
@@ -1838,10 +1838,10 @@
         <v>4205</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
@@ -1849,10 +1849,10 @@
         <v>4210</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
@@ -1871,10 +1871,10 @@
         <v>4220</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
@@ -1882,10 +1882,10 @@
         <v>4225</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -1893,10 +1893,10 @@
         <v>4230</v>
       </c>
       <c r="B49" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
@@ -1904,10 +1904,10 @@
         <v>4235</v>
       </c>
       <c r="B50" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
@@ -1915,10 +1915,10 @@
         <v>4240</v>
       </c>
       <c r="B51" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
@@ -1926,10 +1926,10 @@
         <v>4245</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
@@ -1937,10 +1937,10 @@
         <v>4250</v>
       </c>
       <c r="B53" s="3" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -1948,7 +1948,7 @@
         <v>4255</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C54" s="3" t="n">
         <v>0</v>
@@ -1959,7 +1959,7 @@
         <v>4260</v>
       </c>
       <c r="B55" s="3" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         <v>4270</v>
       </c>
       <c r="B57" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C57" s="3" t="n">
         <v>0</v>
@@ -1992,10 +1992,10 @@
         <v>4275</v>
       </c>
       <c r="B58" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
@@ -2003,7 +2003,7 @@
         <v>4280</v>
       </c>
       <c r="B59" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C59" s="3" t="n">
         <v>0</v>
@@ -2014,7 +2014,7 @@
         <v>4285</v>
       </c>
       <c r="B60" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C60" s="3" t="n">
         <v>0</v>
@@ -2025,7 +2025,7 @@
         <v>4290</v>
       </c>
       <c r="B61" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C61" s="3" t="n">
         <v>0</v>
@@ -2036,7 +2036,7 @@
         <v>4295</v>
       </c>
       <c r="B62" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C62" s="3" t="n">
         <v>0</v>
@@ -2047,10 +2047,10 @@
         <v>4300</v>
       </c>
       <c r="B63" s="3" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="C63" s="3" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
@@ -2058,7 +2058,7 @@
         <v>4305</v>
       </c>
       <c r="B64" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C64" s="3" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>4315</v>
       </c>
       <c r="B66" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C66" s="3" t="n">
         <v>0</v>
@@ -2091,7 +2091,7 @@
         <v>4320</v>
       </c>
       <c r="B67" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C67" s="3" t="n">
         <v>0</v>
@@ -2102,10 +2102,10 @@
         <v>4325</v>
       </c>
       <c r="B68" s="3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2113,7 +2113,7 @@
         <v>4330</v>
       </c>
       <c r="B69" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C69" s="3" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
         <v>4340</v>
       </c>
       <c r="B71" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C71" s="3" t="n">
         <v>0</v>
@@ -2157,10 +2157,10 @@
         <v>4350</v>
       </c>
       <c r="B73" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2212,10 +2212,10 @@
         <v>4375</v>
       </c>
       <c r="B78" s="3" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C78" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2267,10 +2267,10 @@
         <v>4400</v>
       </c>
       <c r="B83" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C83" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2285,444 +2285,204 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="n">
-        <v>4410</v>
-      </c>
-      <c r="B85" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C85" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A85" s="3" t="n"/>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="3" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="n">
-        <v>4415</v>
-      </c>
-      <c r="B86" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C86" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A86" s="3" t="n"/>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="3" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="3" t="n">
-        <v>4420</v>
-      </c>
-      <c r="B87" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C87" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A87" s="3" t="n"/>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="n">
-        <v>4425</v>
-      </c>
-      <c r="B88" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C88" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="A88" s="3" t="n"/>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="3" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="n">
-        <v>4430</v>
-      </c>
-      <c r="B89" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C89" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A89" s="3" t="n"/>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="n">
-        <v>4435</v>
-      </c>
-      <c r="B90" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C90" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A90" s="3" t="n"/>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="3" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="n">
-        <v>4440</v>
-      </c>
-      <c r="B91" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C91" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A91" s="3" t="n"/>
+      <c r="B91" s="3" t="n"/>
+      <c r="C91" s="3" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="n">
-        <v>4445</v>
-      </c>
-      <c r="B92" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C92" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A92" s="3" t="n"/>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="n">
-        <v>4450</v>
-      </c>
-      <c r="B93" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C93" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A93" s="3" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="3" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="n">
-        <v>4455</v>
-      </c>
-      <c r="B94" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C94" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A94" s="3" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="3" t="n">
-        <v>4460</v>
-      </c>
-      <c r="B95" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C95" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A95" s="3" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="3" t="n">
-        <v>4465</v>
-      </c>
-      <c r="B96" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C96" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A96" s="3" t="n"/>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="3" t="n">
-        <v>4470</v>
-      </c>
-      <c r="B97" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C97" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A97" s="3" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="3" t="n">
-        <v>4475</v>
-      </c>
-      <c r="B98" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C98" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A98" s="3" t="n"/>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="3" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="3" t="n">
-        <v>4480</v>
-      </c>
-      <c r="B99" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C99" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A99" s="3" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="3" t="n">
-        <v>4485</v>
-      </c>
-      <c r="B100" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C100" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A100" s="3" t="n"/>
+      <c r="B100" s="3" t="n"/>
+      <c r="C100" s="3" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="3" t="n">
-        <v>4490</v>
-      </c>
-      <c r="B101" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C101" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A101" s="3" t="n"/>
+      <c r="B101" s="3" t="n"/>
+      <c r="C101" s="3" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="n">
-        <v>4495</v>
-      </c>
-      <c r="B102" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C102" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A102" s="3" t="n"/>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="3" t="n">
-        <v>4500</v>
-      </c>
-      <c r="B103" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C103" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A103" s="3" t="n"/>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="n">
-        <v>4505</v>
-      </c>
-      <c r="B104" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C104" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A104" s="3" t="n"/>
+      <c r="B104" s="3" t="n"/>
+      <c r="C104" s="3" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="3" t="n">
-        <v>4510</v>
-      </c>
-      <c r="B105" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A105" s="3" t="n"/>
+      <c r="B105" s="3" t="n"/>
+      <c r="C105" s="3" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="3" t="n">
-        <v>4515</v>
-      </c>
-      <c r="B106" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C106" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A106" s="3" t="n"/>
+      <c r="B106" s="3" t="n"/>
+      <c r="C106" s="3" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="3" t="n">
-        <v>4520</v>
-      </c>
-      <c r="B107" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C107" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A107" s="3" t="n"/>
+      <c r="B107" s="3" t="n"/>
+      <c r="C107" s="3" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="3" t="n">
-        <v>4525</v>
-      </c>
-      <c r="B108" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C108" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A108" s="3" t="n"/>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="3" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="3" t="n">
-        <v>4530</v>
-      </c>
-      <c r="B109" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C109" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A109" s="3" t="n"/>
+      <c r="B109" s="3" t="n"/>
+      <c r="C109" s="3" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="n">
-        <v>4535</v>
-      </c>
-      <c r="B110" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C110" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A110" s="3" t="n"/>
+      <c r="B110" s="3" t="n"/>
+      <c r="C110" s="3" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="3" t="n">
-        <v>4540</v>
-      </c>
-      <c r="B111" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C111" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A111" s="3" t="n"/>
+      <c r="B111" s="3" t="n"/>
+      <c r="C111" s="3" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="3" t="n">
-        <v>4545</v>
-      </c>
-      <c r="B112" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C112" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A112" s="3" t="n"/>
+      <c r="B112" s="3" t="n"/>
+      <c r="C112" s="3" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="n">
-        <v>4550</v>
-      </c>
-      <c r="B113" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C113" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A113" s="3" t="n"/>
+      <c r="B113" s="3" t="n"/>
+      <c r="C113" s="3" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="3" t="n">
-        <v>4555</v>
-      </c>
-      <c r="B114" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C114" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A114" s="3" t="n"/>
+      <c r="B114" s="3" t="n"/>
+      <c r="C114" s="3" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="3" t="n">
-        <v>4560</v>
-      </c>
-      <c r="B115" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C115" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A115" s="3" t="n"/>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="3" t="n">
-        <v>4565</v>
-      </c>
-      <c r="B116" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C116" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A116" s="3" t="n"/>
+      <c r="B116" s="3" t="n"/>
+      <c r="C116" s="3" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="3" t="n">
-        <v>4570</v>
-      </c>
-      <c r="B117" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C117" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A117" s="3" t="n"/>
+      <c r="B117" s="3" t="n"/>
+      <c r="C117" s="3" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="3" t="n">
-        <v>4575</v>
-      </c>
-      <c r="B118" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C118" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A118" s="3" t="n"/>
+      <c r="B118" s="3" t="n"/>
+      <c r="C118" s="3" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="3" t="n">
-        <v>4580</v>
-      </c>
-      <c r="B119" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C119" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A119" s="3" t="n"/>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="3" t="n">
-        <v>4585</v>
-      </c>
-      <c r="B120" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C120" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A120" s="3" t="n"/>
+      <c r="B120" s="3" t="n"/>
+      <c r="C120" s="3" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="3" t="n">
-        <v>4590</v>
-      </c>
-      <c r="B121" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C121" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A121" s="3" t="n"/>
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="3" t="n">
-        <v>4595</v>
-      </c>
-      <c r="B122" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C122" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A122" s="3" t="n"/>
+      <c r="B122" s="3" t="n"/>
+      <c r="C122" s="3" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="3" t="n">
-        <v>4600</v>
-      </c>
-      <c r="B123" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C123" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A123" s="3" t="n"/>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="3" t="n">
-        <v>4605</v>
-      </c>
-      <c r="B124" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C124" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="A124" s="3" t="n"/>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n"/>
@@ -2930,7 +2690,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>2026-09-30 OG1V6 (Week 1 - OCT 2026)</t>
+          <t>2026-10-02 G1TV6 (Week 1 - OCT 2026)</t>
         </is>
       </c>
       <c r="AB1" s="2" t="inlineStr">
@@ -3146,7 +2906,7 @@
         </is>
       </c>
       <c r="J6" s="29" t="n">
-        <v>4186.7</v>
+        <v>4162.3</v>
       </c>
       <c r="AB6">
         <f>IF(NOT(ISNUMBER('Gamma Data'!A6)),"",IF((ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))=0,"",IF(OR(ABS('Gamma Data'!A6-$J$6)&gt;$J$6*$J$26,ABS('Gamma Data'!A6-$J$6)&lt;$J$28),"",(ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))/MAX(ABS('Gamma Data'!A6-$J$6)/($J$6*0.005),1)+ROW()/1000000000)))</f>
@@ -13062,7 +12822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13216,7 +12976,75 @@
         <v>4200</v>
       </c>
       <c r="J4" s="47" t="n">
-        <v>46297.40990339634</v>
+        <v>46297.40990339121</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>G1MV6</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="n">
+        <v>4162.3</v>
+      </c>
+      <c r="D5" s="44" t="n">
+        <v>281</v>
+      </c>
+      <c r="E5" s="44" t="n">
+        <v>339</v>
+      </c>
+      <c r="F5" s="44" t="n">
+        <v>-58</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Negative GEX (แกว่งแรง)</t>
+        </is>
+      </c>
+      <c r="H5" s="44" t="n"/>
+      <c r="I5" s="44" t="n">
+        <v>4170</v>
+      </c>
+      <c r="J5" s="47" t="n">
+        <v>46300.37909289352</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="42" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>G1TV6</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="n">
+        <v>4162.3</v>
+      </c>
+      <c r="D6" s="44" t="n">
+        <v>153</v>
+      </c>
+      <c r="E6" s="44" t="n">
+        <v>209</v>
+      </c>
+      <c r="F6" s="44" t="n">
+        <v>-56</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Negative GEX (แกว่งแรง)</t>
+        </is>
+      </c>
+      <c r="H6" s="44" t="n"/>
+      <c r="I6" s="44" t="n">
+        <v>4175</v>
+      </c>
+      <c r="J6" s="47" t="n">
+        <v>46301.38515448279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Measure GEX levels from the live futures quote; fix flaky Excel read-back
The report's price was the previous session's settle (4,187.1) while the
user's chart (BlackBull gold futures on TradingView) showed ~4,160, so walls,
pins and distances looked wrong. fetch() now also reads CME's own 10-min
delayed quote for the price future (quotes/v2); update_gex writes it to
GEX Calc!J6 and the Log and uses it for Gamma Flip (gex_price_source:
"settle" restores the old behaviour). The card shows the quote time and
the settle next to it. The Max Pain workbook keeps the settle (verify.py
checks it against CME); verify.py recomputes Gamma Flip from the Log price.

verify.excel_cells: Workbooks.Open() returned $null about 1 run in 6 -
retry it; kill exactly the EXCEL.EXE this call started, in finally, so an
error can no longer leak one or touch another run's/the user's Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GEX V.4.1.xlsx
+++ b/GEX V.4.1.xlsx
@@ -3173,7 +3173,7 @@
         </is>
       </c>
       <c r="J6" s="11" t="n">
-        <v>4187.1</v>
+        <v>4158.9</v>
       </c>
       <c r="AB6">
         <f>IF(NOT(ISNUMBER('Gamma Data'!A6)),"",IF((ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))=0,"",IF(OR(ABS('Gamma Data'!A6-$J$6)&gt;$J$6*$J$26,ABS('Gamma Data'!A6-$J$6)&lt;$J$28),"",(ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))/MAX(ABS('Gamma Data'!A6-$J$6)/($J$6*0.005),1)+ROW()/1000000000)))</f>
@@ -13324,7 +13324,7 @@
         </is>
       </c>
       <c r="C7" s="28" t="n">
-        <v>4187.1</v>
+        <v>4158.9</v>
       </c>
       <c r="D7" s="29" t="n">
         <v>317</v>
@@ -13345,7 +13345,7 @@
         <v>4185</v>
       </c>
       <c r="J7" s="42" t="n">
-        <v>46302.53357564853</v>
+        <v>46302.58578933147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
All-expiration GEX, stale-data banner, 11:00 run, J12 fix, WARN vs FAIL
- update_gex_all(): every expiration in QuikStrike's default expiry matrix
  (fetch_gamma.fetch_gamma_all), summed per strike, the workbook's level
  rules applied (levels()); history in a new "Log รวม" sheet; "GEX รวม"
  section on the phone card and in the caption
- card: orange banner when the data is older than the previous weekday
  (CME hadn't published yet); third scheduled run at 11:00 picks it up
- GEX V.4.1.xlsx J12: median gross over strikes with gamma within ±J26 of
  the price (was 0 -> every row "จุดหนืด")
- run_daily.bat: workbook open / GEX skipped is WARN, only a crash or
  non-zero exit is FAIL; run.log rotates past 1 MB
- util.launch_persistent: retry Chrome launch (exited at launch 2026-10-05)
- python_mode delegates to update_gex.mode_label (one copy of the rule)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GEX V.4.1.xlsx
+++ b/GEX V.4.1.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEX Calc" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บันทึกโหมด" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log รวม" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -18,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="0.0\×"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="\+#,##0;\-#,##0;0"/>
@@ -31,6 +32,7 @@
     <numFmt numFmtId="173" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="174" formatCode="yyyy-mm-dd hh:mm"/>
     <numFmt numFmtId="175" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="176" formatCode="0.000"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -229,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -309,6 +311,7 @@
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -506,7 +509,7 @@
           </dLbls>
           <cat>
             <numRef>
-              <f>'GEX Calc'!$A$2:$A$109</f>
+              <f>'GEX Calc'!$A$2:$A$104</f>
               <numCache>
                 <formatCode>#,##0</formatCode>
                 <ptCount val="83"/>
@@ -764,7 +767,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'GEX Calc'!$C$2:$C$109</f>
+              <f>'GEX Calc'!$C$2:$C$104</f>
               <numCache>
                 <formatCode>#,##0</formatCode>
                 <ptCount val="83"/>
@@ -1490,7 +1493,7 @@
     </row>
     <row r="2" ht="15" customHeight="1" s="35">
       <c r="A2" s="2" t="n">
-        <v>4095</v>
+        <v>3995</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>0</v>
@@ -1501,18 +1504,18 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="35">
       <c r="A3" s="2" t="n">
-        <v>4100</v>
+        <v>4000</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="35">
       <c r="A4" s="2" t="n">
-        <v>4105</v>
+        <v>4005</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0</v>
@@ -1523,40 +1526,40 @@
     </row>
     <row r="5" ht="15" customHeight="1" s="35">
       <c r="A5" s="2" t="n">
-        <v>4110</v>
+        <v>4010</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="35">
       <c r="A6" s="2" t="n">
-        <v>4115</v>
+        <v>4015</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="35">
       <c r="A7" s="2" t="n">
-        <v>4120</v>
+        <v>4020</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="35">
       <c r="A8" s="2" t="n">
-        <v>4125</v>
+        <v>4025</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0</v>
@@ -1567,260 +1570,260 @@
     </row>
     <row r="9" ht="15" customHeight="1" s="35">
       <c r="A9" s="2" t="n">
-        <v>4130</v>
+        <v>4030</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="35">
       <c r="A10" s="2" t="n">
-        <v>4135</v>
+        <v>4035</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="35">
       <c r="A11" s="2" t="n">
-        <v>4140</v>
+        <v>4040</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="35">
       <c r="A12" s="2" t="n">
-        <v>4145</v>
+        <v>4045</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="35">
       <c r="A13" s="2" t="n">
-        <v>4150</v>
+        <v>4050</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>18</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="35">
       <c r="A14" s="2" t="n">
-        <v>4155</v>
+        <v>4055</v>
       </c>
       <c r="B14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>19</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="35">
       <c r="A15" s="2" t="n">
-        <v>4160</v>
+        <v>4060</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="35">
       <c r="A16" s="2" t="n">
-        <v>4165</v>
+        <v>4065</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="35">
       <c r="A17" s="2" t="n">
-        <v>4170</v>
+        <v>4070</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="35">
       <c r="A18" s="2" t="n">
-        <v>4175</v>
+        <v>4075</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="35">
       <c r="A19" s="2" t="n">
-        <v>4180</v>
+        <v>4080</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="35">
       <c r="A20" s="2" t="n">
-        <v>4185</v>
+        <v>4085</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>57</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="35">
       <c r="A21" s="2" t="n">
-        <v>4190</v>
+        <v>4090</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="35">
       <c r="A22" s="2" t="n">
-        <v>4195</v>
+        <v>4095</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="35">
       <c r="A23" s="2" t="n">
-        <v>4200</v>
+        <v>4100</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>23</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="35">
       <c r="A24" s="2" t="n">
-        <v>4205</v>
+        <v>4105</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="35">
       <c r="A25" s="2" t="n">
-        <v>4210</v>
+        <v>4110</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="35">
       <c r="A26" s="2" t="n">
-        <v>4215</v>
+        <v>4115</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="35">
       <c r="A27" s="2" t="n">
-        <v>4220</v>
+        <v>4120</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="35">
       <c r="A28" s="2" t="n">
-        <v>4225</v>
+        <v>4125</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="35">
       <c r="A29" s="2" t="n">
-        <v>4230</v>
+        <v>4130</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="35">
       <c r="A30" s="2" t="n">
-        <v>4235</v>
+        <v>4135</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="35">
       <c r="A31" s="2" t="n">
-        <v>4240</v>
+        <v>4140</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="35">
       <c r="A32" s="2" t="n">
-        <v>4245</v>
+        <v>4145</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>2</v>
@@ -1831,142 +1834,142 @@
     </row>
     <row r="33" ht="15" customHeight="1" s="35">
       <c r="A33" s="2" t="n">
-        <v>4250</v>
+        <v>4150</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>5</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="35">
       <c r="A34" s="2" t="n">
-        <v>4255</v>
+        <v>4155</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="35">
       <c r="A35" s="2" t="n">
-        <v>4260</v>
+        <v>4160</v>
       </c>
       <c r="B35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="35">
       <c r="A36" s="2" t="n">
-        <v>4265</v>
+        <v>4165</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="35">
       <c r="A37" s="2" t="n">
-        <v>4270</v>
+        <v>4170</v>
       </c>
       <c r="B37" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="35">
       <c r="A38" s="2" t="n">
-        <v>4275</v>
+        <v>4175</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="35">
       <c r="A39" s="2" t="n">
-        <v>4280</v>
+        <v>4180</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="35">
       <c r="A40" s="2" t="n">
-        <v>4285</v>
+        <v>4185</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="35">
       <c r="A41" s="2" t="n">
-        <v>4290</v>
+        <v>4190</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="35">
       <c r="A42" s="2" t="n">
-        <v>4295</v>
+        <v>4195</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="35">
       <c r="A43" s="2" t="n">
-        <v>4300</v>
+        <v>4200</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="35">
       <c r="A44" s="2" t="n">
-        <v>4305</v>
+        <v>4205</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="35">
       <c r="A45" s="2" t="n">
-        <v>4310</v>
+        <v>4210</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
@@ -1974,10 +1977,10 @@
     </row>
     <row r="46" ht="15" customHeight="1" s="35">
       <c r="A46" s="2" t="n">
-        <v>4315</v>
+        <v>4215</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C46" s="2" t="n">
         <v>0</v>
@@ -1985,10 +1988,10 @@
     </row>
     <row r="47" ht="15" customHeight="1" s="35">
       <c r="A47" s="2" t="n">
-        <v>4320</v>
+        <v>4220</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C47" s="2" t="n">
         <v>0</v>
@@ -1996,21 +1999,21 @@
     </row>
     <row r="48" ht="15" customHeight="1" s="35">
       <c r="A48" s="2" t="n">
-        <v>4325</v>
+        <v>4225</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="35">
       <c r="A49" s="2" t="n">
-        <v>4330</v>
+        <v>4230</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C49" s="2" t="n">
         <v>0</v>
@@ -2018,10 +2021,10 @@
     </row>
     <row r="50" ht="15" customHeight="1" s="35">
       <c r="A50" s="2" t="n">
-        <v>4335</v>
+        <v>4235</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" s="2" t="n">
         <v>0</v>
@@ -2029,10 +2032,10 @@
     </row>
     <row r="51" ht="15" customHeight="1" s="35">
       <c r="A51" s="2" t="n">
-        <v>4340</v>
+        <v>4240</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51" s="2" t="n">
         <v>0</v>
@@ -2040,10 +2043,10 @@
     </row>
     <row r="52" ht="15" customHeight="1" s="35">
       <c r="A52" s="2" t="n">
-        <v>4345</v>
+        <v>4245</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>0</v>
@@ -2051,21 +2054,21 @@
     </row>
     <row r="53" ht="15" customHeight="1" s="35">
       <c r="A53" s="2" t="n">
-        <v>4350</v>
+        <v>4250</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="35">
       <c r="A54" s="2" t="n">
-        <v>4355</v>
+        <v>4255</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2" t="n">
         <v>0</v>
@@ -2073,10 +2076,10 @@
     </row>
     <row r="55" ht="15" customHeight="1" s="35">
       <c r="A55" s="2" t="n">
-        <v>4360</v>
+        <v>4260</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>0</v>
@@ -2084,10 +2087,10 @@
     </row>
     <row r="56" ht="15" customHeight="1" s="35">
       <c r="A56" s="2" t="n">
-        <v>4365</v>
+        <v>4265</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C56" s="2" t="n">
         <v>0</v>
@@ -2095,7 +2098,7 @@
     </row>
     <row r="57" ht="15" customHeight="1" s="35">
       <c r="A57" s="2" t="n">
-        <v>4370</v>
+        <v>4270</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>0</v>
@@ -2106,21 +2109,21 @@
     </row>
     <row r="58" ht="15" customHeight="1" s="35">
       <c r="A58" s="2" t="n">
-        <v>4375</v>
+        <v>4275</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="35">
       <c r="A59" s="2" t="n">
-        <v>4380</v>
+        <v>4280</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C59" s="2" t="n">
         <v>0</v>
@@ -2128,10 +2131,10 @@
     </row>
     <row r="60" ht="15" customHeight="1" s="35">
       <c r="A60" s="2" t="n">
-        <v>4385</v>
+        <v>4285</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C60" s="2" t="n">
         <v>0</v>
@@ -2139,10 +2142,10 @@
     </row>
     <row r="61" ht="15" customHeight="1" s="35">
       <c r="A61" s="2" t="n">
-        <v>4390</v>
+        <v>4290</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C61" s="2" t="n">
         <v>0</v>
@@ -2150,7 +2153,7 @@
     </row>
     <row r="62" ht="15" customHeight="1" s="35">
       <c r="A62" s="2" t="n">
-        <v>4395</v>
+        <v>4295</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>0</v>
@@ -2161,18 +2164,18 @@
     </row>
     <row r="63" ht="15" customHeight="1" s="35">
       <c r="A63" s="2" t="n">
-        <v>4400</v>
+        <v>4300</v>
       </c>
       <c r="B63" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C63" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="35">
       <c r="A64" s="2" t="n">
-        <v>4405</v>
+        <v>4305</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>0</v>
@@ -2183,7 +2186,7 @@
     </row>
     <row r="65" ht="15" customHeight="1" s="35">
       <c r="A65" s="2" t="n">
-        <v>4410</v>
+        <v>4310</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>0</v>
@@ -2194,7 +2197,7 @@
     </row>
     <row r="66" ht="15" customHeight="1" s="35">
       <c r="A66" s="2" t="n">
-        <v>4415</v>
+        <v>4315</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>0</v>
@@ -2205,7 +2208,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>4420</v>
+        <v>4320</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>0</v>
@@ -2216,21 +2219,21 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>4425</v>
+        <v>4325</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>4430</v>
+        <v>4330</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C69" s="2" t="n">
         <v>0</v>
@@ -2238,7 +2241,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>4435</v>
+        <v>4335</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>0</v>
@@ -2249,7 +2252,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>4440</v>
+        <v>4340</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>0</v>
@@ -2260,7 +2263,7 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>4445</v>
+        <v>4345</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>0</v>
@@ -2271,10 +2274,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>4450</v>
+        <v>4350</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C73" s="2" t="n">
         <v>0</v>
@@ -2282,7 +2285,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>4455</v>
+        <v>4355</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>0</v>
@@ -2293,7 +2296,7 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>4460</v>
+        <v>4360</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>0</v>
@@ -2304,7 +2307,7 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>4465</v>
+        <v>4365</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>0</v>
@@ -2315,7 +2318,7 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>4470</v>
+        <v>4370</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>0</v>
@@ -2326,10 +2329,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>4475</v>
+        <v>4375</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C78" s="2" t="n">
         <v>0</v>
@@ -2337,7 +2340,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>4480</v>
+        <v>4380</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>0</v>
@@ -2348,7 +2351,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>4485</v>
+        <v>4385</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>0</v>
@@ -2359,7 +2362,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>4490</v>
+        <v>4390</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>0</v>
@@ -2370,7 +2373,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>4495</v>
+        <v>4395</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>0</v>
@@ -2381,10 +2384,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>4500</v>
+        <v>4400</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C83" s="2" t="n">
         <v>0</v>
@@ -2392,7 +2395,7 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>4505</v>
+        <v>4405</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>0</v>
@@ -2403,7 +2406,7 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>4510</v>
+        <v>4410</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>0</v>
@@ -2414,7 +2417,7 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>4515</v>
+        <v>4415</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>0</v>
@@ -2425,7 +2428,7 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>4520</v>
+        <v>4420</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>0</v>
@@ -2436,10 +2439,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>4525</v>
+        <v>4425</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C88" s="2" t="n">
         <v>0</v>
@@ -2447,7 +2450,7 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>4530</v>
+        <v>4430</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>0</v>
@@ -2458,7 +2461,7 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>4535</v>
+        <v>4435</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>0</v>
@@ -2469,7 +2472,7 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>4540</v>
+        <v>4440</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>0</v>
@@ -2480,7 +2483,7 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>4545</v>
+        <v>4445</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>0</v>
@@ -2491,10 +2494,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>4550</v>
+        <v>4450</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C93" s="2" t="n">
         <v>0</v>
@@ -2502,7 +2505,7 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>4555</v>
+        <v>4455</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>0</v>
@@ -2513,7 +2516,7 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>4560</v>
+        <v>4460</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>0</v>
@@ -2524,7 +2527,7 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>4565</v>
+        <v>4465</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>0</v>
@@ -2535,7 +2538,7 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>4570</v>
+        <v>4470</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>0</v>
@@ -2546,10 +2549,10 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>4575</v>
+        <v>4475</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C98" s="2" t="n">
         <v>0</v>
@@ -2557,7 +2560,7 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>4580</v>
+        <v>4480</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>0</v>
@@ -2568,7 +2571,7 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>4585</v>
+        <v>4485</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>0</v>
@@ -2579,7 +2582,7 @@
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>4590</v>
+        <v>4490</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>0</v>
@@ -2590,7 +2593,7 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>4595</v>
+        <v>4495</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>0</v>
@@ -2601,7 +2604,7 @@
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>4600</v>
+        <v>4500</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>1</v>
@@ -2612,7 +2615,7 @@
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>4605</v>
+        <v>4505</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>0</v>
@@ -2622,59 +2625,29 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
-        <v>4610</v>
-      </c>
-      <c r="B105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A105" s="2" t="n"/>
+      <c r="B105" s="2" t="n"/>
+      <c r="C105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
-        <v>4615</v>
-      </c>
-      <c r="B106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C106" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A106" s="2" t="n"/>
+      <c r="B106" s="2" t="n"/>
+      <c r="C106" s="2" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
-        <v>4620</v>
-      </c>
-      <c r="B107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C107" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A107" s="2" t="n"/>
+      <c r="B107" s="2" t="n"/>
+      <c r="C107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
-        <v>4625</v>
-      </c>
-      <c r="B108" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C108" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A108" s="2" t="n"/>
+      <c r="B108" s="2" t="n"/>
+      <c r="C108" s="2" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
-        <v>4650</v>
-      </c>
-      <c r="B109" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C109" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A109" s="2" t="n"/>
+      <c r="B109" s="2" t="n"/>
+      <c r="C109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -2957,7 +2930,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>2026-10-06 G1WV6 (Week 1 - OCT 2026)</t>
+          <t>2026-10-07 OG2V6 (Week 2 - OCT 2026)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -3173,7 +3146,7 @@
         </is>
       </c>
       <c r="J6" s="11" t="n">
-        <v>4158.9</v>
+        <v>4199.1</v>
       </c>
       <c r="AB6">
         <f>IF(NOT(ISNUMBER('Gamma Data'!A6)),"",IF((ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))=0,"",IF(OR(ABS('Gamma Data'!A6-$J$6)&gt;$J$6*$J$26,ABS('Gamma Data'!A6-$J$6)&lt;$J$28),"",(ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))/MAX(ABS('Gamma Data'!A6-$J$6)/($J$6*0.005),1)+ROW()/1000000000)))</f>
@@ -3417,11 +3390,11 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>ค่ากลาง Gross</t>
+          <t>ค่ากลาง Gross (strike ที่มี gamma, ±J26 ของราคา)</t>
         </is>
       </c>
       <c r="J12" s="15">
-        <f t="array" ref="J12">MEDIAN(IF(ISNUMBER('Gamma Data'!$A$2:$A$152),ABS('Gamma Data'!$B$2:$B$152)+ABS('Gamma Data'!$C$2:$C$152)))</f>
+        <f t="array" ref="J12">IFERROR(MEDIAN(IF(ISNUMBER('Gamma Data'!$A$2:$A$152)*((ABS('Gamma Data'!$B$2:$B$152)+ABS('Gamma Data'!$C$2:$C$152))&gt;0)*(ABS('Gamma Data'!$A$2:$A$152-$J$6)&lt;=$J$6*$J$26),(ABS('Gamma Data'!$B$2:$B$152)+ABS('Gamma Data'!$C$2:$C$152)))),0)</f>
         <v/>
       </c>
       <c r="AB12">
@@ -13089,7 +13062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13345,7 +13318,233 @@
         <v>4185</v>
       </c>
       <c r="J7" s="42" t="n">
-        <v>46302.58578933147</v>
+        <v>46302.5857893287</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>G2RV6</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>4157.9</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>132</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>185</v>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>-53</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Negative GEX (แกว่งแรง)</t>
+        </is>
+      </c>
+      <c r="H8" s="29" t="n"/>
+      <c r="I8" s="29" t="n">
+        <v>4200</v>
+      </c>
+      <c r="J8" s="42" t="n">
+        <v>46303.37572651621</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>G2RV6</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>4149.9</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>369</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>418</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>-49</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Negative GEX (แกว่งแรง)</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="n"/>
+      <c r="I9" s="29" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J9" s="42" t="n">
+        <v>46303.58431898148</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="40" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>OG2V6</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>4199.1</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>391</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>640</v>
+      </c>
+      <c r="F10" s="29" t="n">
+        <v>-249</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Negative GEX (แกว่งแรง)</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="n"/>
+      <c r="I10" s="29" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J10" s="42" t="n">
+        <v>46304.43079458334</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>วันที่ข้อมูล</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>สัญญาที่รวม</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ราคา</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>รวม Call Gamma</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>รวม Put Gamma</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>NET GEX</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>โหมด</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Conviction</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Call Wall</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Put Wall</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Gamma Flip</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Strike gamma สูงสุด</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>บันทึกเมื่อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>OG2V6, OGX6, OGZ6, OGF7, OGG7, OGH7, OGJ7, OGM7, OGQ7</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="n">
+        <v>4199.1</v>
+      </c>
+      <c r="D2" s="29" t="n">
+        <v>6755</v>
+      </c>
+      <c r="E2" s="29" t="n">
+        <v>7034</v>
+      </c>
+      <c r="F2" s="29" t="n">
+        <v>-279</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ไม่มีโหมด</t>
+        </is>
+      </c>
+      <c r="H2" s="43" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="I2" s="29" t="n">
+        <v>4500</v>
+      </c>
+      <c r="J2" s="29" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K2" s="29" t="n"/>
+      <c r="L2" s="29" t="n">
+        <v>4100</v>
+      </c>
+      <c r="M2" s="42" t="n">
+        <v>46304.43123911203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>